<commit_message>
13-05-25 (2) Joanny la dernière personne
</commit_message>
<xml_diff>
--- a/bd1.xlsx
+++ b/bd1.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M74"/>
+  <dimension ref="A1:M100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4024,10 +4024,8 @@
           <t>KOUASSI Louis Gerard</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>0102989154</t>
-        </is>
+      <c r="E70" t="n">
+        <v>102989154</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -4130,10 +4128,8 @@
           <t>KONAN  Atse Franck Désiré</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>0787347707</t>
-        </is>
+      <c r="E72" t="n">
+        <v>787347707</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -4183,10 +4179,8 @@
           <t>MOBIO Adja Axel Prince Yvon</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>0141583425</t>
-        </is>
+      <c r="E73" t="n">
+        <v>141583425</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -4236,10 +4230,8 @@
           <t>KONE Alligué Samirah Angela Mauricette</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>0758422493</t>
-        </is>
+      <c r="E74" t="n">
+        <v>758422493</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -4269,6 +4261,1330 @@
       </c>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>44944</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>DOUCOURE</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Oumou</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>DOUCOURE Oumou</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Analyse de la gestion du risque inhérent à l'octroi de crédit bancaire aux entreprises: cas de la Banque Populaire de Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Banque populaire</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>N'GUESSA Simon Pierre</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>44945</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>NIAMKE</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Ahdjey David Loic Emmanuel</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>NIAMKE Ahdjey David Loic Emmanuel</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Effet de l'ouverture commercial et des flux de capitaux sur la croissance économique en Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Economie de développement</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Economie de développement</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Economie de développement</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>AKA Brou Emmanuel</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>44945</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>BENIAMBIE</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Aka Ephraim Herman</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>BENIAMBIE Aka Ephraim Herman</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Mise en place d'un manuel de procédure de gestion de trésorie</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>N'GUESSA Simon Pierre</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>44946</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>TRAORE</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>BINTA</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>TRAORE BINTA</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>L'évaluation du contrôle interne d'une entreprise de distribution d'un service financier numérique</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>FOFANA Andom</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>44844</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>BAOUNA</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Domo</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>BAOUNA Domo</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Analyse des effets du commerce international sur la sécurité alimentaire des ménages: cas des ménages du Tchad</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>KONE Salif</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>44952</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>OUATTARA</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Kra</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>OUATTARA Kra</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Impact des dépenses publiques sociales sur la croissance économique en CI</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>KOUAKOU Auguste</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>44620</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>OUATTARA</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Abdel Kader</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>OUATTARA Abdel Kader</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Contribution à l'amélioration de l'élaboration des états financiers des entités dans le cadre de la mission de visa</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>FOFANA Adom</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>44957</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>TANOE</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Ahoba Marie-Déirée</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>TANOE Ahoba Marie-Déirée</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>767469615</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Contribution de la revision comptable à la gestion financières et comptable d'une entreprise; cas de COMTRATS</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>COMTRATS</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>FOFANA Andom</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>45013</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>BLE</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Israel Djedje</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>BLE Israel Djedje</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>La fiscalité comme lévier de développement: cas de la Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>MOUSSA Kouame Richard</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>45013</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>ATTA</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>N'Doua Jean Christian</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>ATTA N'Doua Jean Christian</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Analyse des facteurs limitant la production des éléveurs de porcs de la ville d'Abidjan et ses alentours</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>MOUSSA Kouame Richard</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>45386</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>LAGO</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Logblo Olga-Dominique</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>LAGO Logblo Olga-Dominique</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Analyse de stratégie de fidélisation des clients de la banque des dépôts du trésor public de Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Banque et assurane</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Banque et assurane</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Banque du trésor</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>SANGARE Tchetien</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>45103</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>KOUKONI</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Gloria Marina</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>KOUKONI Gloria Marina</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Conquête et fidélisation de la clientèle, un jeu pour les banques aujour'hui: Cas de la BHCI</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>BHCI</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>APKESSE</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>45107</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>TRAORE</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Cadic Laeticia Ley</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>TRAORE Cadic Laeticia Ley</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Finances islamique et inclusion financière</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>MOUSSA Kouamé Richard</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>45107</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>AVY</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Sombo Marie-Andrée Eugenie</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>AVY Sombo Marie-Andrée Eugenie</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Fracture numérique et transition démographique en Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>KOUAKOU Auguste</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>45107</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>TIAPANI</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Akpa Jean Cyriaque</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>TIAPANI Akpa Jean Cyriaque</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Impact de la COVID-19 sur le commerce électronique en Afrique cas de Jumia</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>KOUAKOU Auguste</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>45107</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>BAMBA</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Awa</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>BAMBA Awa</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>La mission du commissaire aux comptes dans la certification du cycle vente-client: cas de la société X</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>SANGARE</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>45107</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>OSSEY</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Reine Marina Aude</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>OSSEY Reine Marina Aude</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Contribution de la mise en oeuvre des recommandations d'audit interne à l'amélioration du processus de gestion des stocks au BNETD</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>BNETD</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>FOFANA Adom</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>45107</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>KOTTY</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Kotty Paul Marie</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>KOTTY Kotty Paul Marie</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Analyse du marché de la téléphonie mobile en Côte d'Ivoire:dynamique du marché et performance des opérateurs</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Sangare Tchetien</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>45110</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>ABIE</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Jeanne</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>ABIE Jeanne</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Analyse de la mission d'audit des dépenses d'alimentation dans l'administrationn publique: cas du centre régionale des oeuvres Universitaires</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>CROU</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Sangare Tchetien</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>45110</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>COULIBALY</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Myriam</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>COULIBALY Myriam</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Analyse des risques liés à la gestion du cycle achats fournisseurs dans le cadre d'une mission de CAC: Cas de l'agence TS Immobilier</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>TS Immobilier</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Fofana César</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>45110</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>KOBRON</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Ehien</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>KOBRON Ehien</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Evolution de la satisfaction clientèle particuluier à l'offre bancaire de prêt immobilier: Cas de la BHCI</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>BHCI</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>KOUASSI Rufin Cyriaque</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>45110</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>DAGRI</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Fleure</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>DAGRI Fleure</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Audit du dispositif HSE: cas du BNETD</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>BNETD</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>FOFANA Andom</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>45110</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>ACHO</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Bah Marie Otnielle</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>ACHO Bah Marie Otnielle</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Impact du contrôle interne sur la performance financière de l'entreprise: Cas du BNETD</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>BNETD</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>FOFANA Andom</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>45110</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>APKA</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Agnimel Claude Virgile</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>APKA Agnimel Claude Virgile</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Evaluation du contrôle interne du Cycle Achat: Cas de VOLCAGRO-CI</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>VOLCAGRO-CI</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>FOFANA Andom</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>45110</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>DOGBO</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Bisso Gilles Kevine</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>DOGBO Bisso Gilles Kevine</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>L'impact du crédit-bail sur la performance financière: Cas de la BICICI</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>BICICI</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>KOUASSI Rufin Cyriaque</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>45110</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>JOANNY</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Tape Waissa Mamita</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>JOANNY Tape Waissa Mamita</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Evaluation des procédures du contrôle interne du cycle Achat/Fournisseur dans le cadre d'une mission de CAC: Cas de la SIA</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>FOFANA Andom</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
14/05/25 (ELEMEHA Danielle Esther)
</commit_message>
<xml_diff>
--- a/bd1.xlsx
+++ b/bd1.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M100"/>
+  <dimension ref="A1:M126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5586,6 +5586,1336 @@
       <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr"/>
     </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>45111</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>DOMANDE</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Satyogo</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>DOMANDE Satyogo</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Evaluation du contrôle interne cycle vente client lors d'une mission d'audit externe: cas de la société alpha</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>BNETD</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>BADINI</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>45112</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>DON</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Boimin Held</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>DON Boimin Held</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>La mise en place du dispositif de contrôle interne au sein d'une société de production de boissons alcoolisées: Cas du département - productions MIBEM-MIB</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>MIBEM-MIB</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>BADINI</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n">
+        <v>45113</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>GLOPKOR</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Ahoefa Dédé Géorgette</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>GLOPKOR Ahoefa Dédé Géorgette</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>L'effet de la fracture numérique sur la sécurité alimentaire en afrique subsaharienne</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Kouakou Auguste</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n">
+        <v>45116</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>KIPRE</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Prince Donald</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>KIPRE Prince Donald</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Transition énergétique en Côte d'Ivoire: L'énergie éolienne, une alternative dans le mix-énergétique</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>ASSOUMOU Ella</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr"/>
+      <c r="M104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n">
+        <v>45240</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>DADIE</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Dogo Jérôme</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>DADIE Dogo Jérôme</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Effet de la corruption sur la croissance économique dans les pays en développement: cas de L'UEMOA</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>ASSOUMOU Ella</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr"/>
+      <c r="M105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>45240</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>KOFFI</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Adamoh Yves Christian</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>KOFFI Adamoh Yves Christian</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Optimisation des délais de traitement de sinistre pour les produits de prévoyance cas WAFA Assurance vie</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Banque et assurane</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Banque et assurane</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>WAFA Assurance</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>NOE Coulibay</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr"/>
+      <c r="M106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>45240</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>ABBY</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Gah Malika</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>ABBY Gah Malika</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Analyse des déterminants de l'acceptabilité des procédures de développement administratifs en ligne par les ivoiriens d'abidjan et ses alentours</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>KOUAKOU Auguste</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr"/>
+      <c r="M107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>45296</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>GOLOT</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Gah Octavie</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>GOLOT Gah Octavie</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Analyse des coûts d'exploitation des véhicules: cas de l'unité agricole intégré d'EHANIA</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>EHANIA</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>FOFANA Adom</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr"/>
+      <c r="M108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>45385</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>SIMDAYIKE</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Cyriaque</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>SIMDAYIKE Cyriaque</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Les mécanismes de mise en place optimale d'un cycle de vie du crédit dans une SFD en Côte d'Ivoire: Cas de DIFIM SA</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Banque et assurane</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Banque et assurane</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>DIFIM SA</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>KOUASSI Rufin</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr"/>
+      <c r="M109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>45385</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>AFFIAN</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Astride Lynda Ama</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>AFFIAN Astride Lynda Ama</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Diagnostic qualité des missions d'assistance comptable au sein du Cabinet 3C</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>3C</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>N'DRI Yachine</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr"/>
+      <c r="M110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>45385</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>LOUA</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Dervine Anne Elisabeth Gausseu</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>LOUA Dervine Anne Elisabeth Gausseu</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>L'accessibilité des PME aux financement du marché par les banques: cas de la banque populaire de Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Banque et assurane</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Banque et assurane</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>banque populaire</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>N'DRI Yachine</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr"/>
+      <c r="M111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>45385</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>FANNY</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Inza Ladji Habib</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>FANNY Inza Ladji Habib</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Effet de la gouvernance sur la croissance économique en Afrique</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>MOUSSA Kouamé Richard</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr"/>
+      <c r="M112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>45385</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>SORO</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Kinignari Zakaria</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>SORO Kinignari Zakaria</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Analyse des déterminants des stratégies d'adaptations des riziculteurs face au changements climatique: un exemple de la région du Kabadougou</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Salif Koné</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr"/>
+      <c r="M113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>45385</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>CAMINO</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Tanobla Morisson</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>CAMINO Tanobla Morisson</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>L'influence de la GRC sur la performance financière de la banque: cas de la SIB</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>SANGARE</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr"/>
+      <c r="M114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n">
+        <v>45385</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>EKOU</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Tanoh Yves Elfried</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>EKOU Tanoh Yves Elfried</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Impact du commerce international sur la croissance économique: Rôle de la corruption en Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>KONE Salif</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr"/>
+      <c r="M115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>45385</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>SACOH</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Dorcas</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>SACOH Dorcas</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Effets des chocs conjoncturelles sur la banlance commerciale des pays de la CEDEAO</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>ASSOUMOU Ella</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr"/>
+      <c r="M116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>45386</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>COULIBALY</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Siombin Nangoti Ali</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>COULIBALY Siombin Nangoti Ali</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Contribution de la cellule de remediaton a la mise à jour des données clientèles: Cas de la Bridge Bank Group Ci</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Bridge Bank</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>SANGARE Tchetchien</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr"/>
+      <c r="M117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>45386</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Agui</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Emmanuella</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Agui Emmanuella</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Amélioration de la satisfaction client dans les établissements bancaires: cas de la BHCI Treichville</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>BHCI</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>Sangare Tchetien</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>45386</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>ABIE</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Jeanne</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>ABIE Jeanne</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Analyse de la mission d'audit des dépenses d'alimentation dans l'administrationn publique: cas du centre régionale des oeuvres Universitaires</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>CROU</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>Sangare Tchetien</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr"/>
+      <c r="M119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>45386</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>KOUADIO</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Aguely Jean</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>KOUADIO Aguely Jean</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Evaluation des risques dans une société de Gestion Immoilière: Une approche d'audit pour la prévention et la détection des risques de fraudes dans la société Beta</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Fofana César</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr"/>
+      <c r="M120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n">
+        <v>45386</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>TRAORE</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Chintchon Aminata</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>TRAORE Chintchon Aminata</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Contribution du contrôle interne à l'amélioration de la gestion des risques opérationnelles: cas de l'entreprise alpha</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>SANGARE Tchétien</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr"/>
+      <c r="M121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n">
+        <v>45387</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>ADJEHI</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>N'Tah Carine</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>ADJEHI N'Tah Carine</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Contribution de l'audit légal à la performance organisationnelle et financière des entreprises: Cas de la société HAMA</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Audit et contrôle</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>HAMA</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>FOFANA Adom</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n">
+        <v>45394</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>AHOUTY</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Tekia</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>AHOUTY Tekia</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Impact des investissements directs étrangers sur l'environnement en Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>économie du développement</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>KOUADIO Benié</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr"/>
+      <c r="M123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n">
+        <v>45469</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>ZANKOU</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Nathalie</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>ZANKOU Nathalie</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Contribution de la gestion des risques organisationnels à la bonne gouvernance des institutions: Cas de CARITAS CI</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Banque et assurane</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Banque et assurane</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>CARITAS CI</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>SANGARE Tchetien</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr"/>
+      <c r="M124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n">
+        <v>45481</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>KOMENAN</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Jean Marie Vianey</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>KOMENAN Jean Marie Vianey</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>La commercialisation des produits dans une micro-assurance: cas de l'UNACOOPEC-CI</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Banque et assurane</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Banque et assurane</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>DOMOA Danielle</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>45483</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>DIOKE Djedjoro</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Djedjoro Antoinnette</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>DIOKE Djedjoro Antoinnette</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>0779968672</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Impact de la digitalisation des produits et services bancaires sur la relation client: Cas de BOA-CI</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Banque et assurance</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Banque et assurane</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Banque et assurane</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>BOA-CI</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>N'DRI Yachine</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>